<commit_message>
some updates for validation
</commit_message>
<xml_diff>
--- a/Scripts/Testing/Genetic_algorithm_tests/Results/toy_model_parametrization.xlsx
+++ b/Scripts/Testing/Genetic_algorithm_tests/Results/toy_model_parametrization.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0051</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.863125958156862</v>
+        <v>1.352203600163681</v>
       </c>
     </row>
     <row r="3">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9727205942395488</v>
+        <v>0.08644916314895364</v>
       </c>
     </row>
     <row r="4">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9308227231670749</v>
+        <v>0.1793596360735628</v>
       </c>
     </row>
   </sheetData>
@@ -687,11 +687,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.02193281536987507</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1.758856798266161,0.5,0.9368261252933587</t>
+          <t>2.8924638724579337,0.569524159734011,1.6708405900886545</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -700,11 +700,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.02193281536987507</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2.002952701827223,0.9202533330178355,0.8544848739988928</t>
+          <t>3.051938536522032,0.569524159734011,4.475213211331274</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -713,11 +713,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.02193281536987507</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2.069301260940083,0.5,0.8988418782812009</t>
+          <t>3.848845395901783,1.4365499502385757,0.20217472269133435</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -726,11 +726,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.02180584918342432</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1,0.9703358629579736,0.8401295290106658</t>
+          <t>1.987646918070706,0.2541695329592857,0.017097034978287927</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -739,11 +739,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.02180584918342432</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.9787274406982085,1.1164733075328155,0.8823294479477539</t>
+          <t>3.0062370479940266,0.0017002151129185455,0.08451912524871687</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -752,11 +752,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.02180584918342432</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.7510076414407258,1.0418027913538919,0.8912426465942411</t>
+          <t>1.2787626029336818,0.19496244078662248,1.4950900680884687</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -765,11 +765,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.02180584918342432</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.8882761518237476,1.0487302555589513,0.9194785218382209</t>
+          <t>0.5402939795689649,0.020983948799077404,0.27806590837091927</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -778,11 +778,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.02180584918342432</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1.9673131741338568,1.0317904426394175,0.8767427550151374</t>
+          <t>0.7392657256664663,2.4734802075819955,0.0030627848696714974</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -791,11 +791,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.02180584918342432</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2.0897849394244927,0.9788964731977542,0.871621460223039</t>
+          <t>1.275396514892563,0.4782933443632343,3.0964047138813497</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -804,11 +804,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.02180584918342432</v>
+        <v>0.03082930686377845</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1,0.9703358629579736,0.8401295290106658</t>
+          <t>0.3817751388303598,0.01649286043169756,1.985586888796016</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -817,11 +817,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.02178692856264347</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1.8554216744384444,0.5,0.9054163731804166</t>
+          <t>0.4828720420349909,0.14892421624637012,0.2783129012578397</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -830,11 +830,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.02178692856264347</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1,0.5,0.9162495827319155</t>
+          <t>1.4324850413658867,0.0002021472584592835,0.02950125796447201</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -843,11 +843,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.02178692856264347</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1,1.0685544403211764,0.9280463430678121</t>
+          <t>0.365644485548155,1.3330180608434845,0.11536738791278571</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -856,11 +856,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.02178692856264347</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2.0799864236490704,0.9538647943932738,0.8863103755483714</t>
+          <t>1.4341642450747463,0.0033107260580177134,0.00025270797536693275</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -869,11 +869,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.02178692856264347</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1,0.5,0.8374157555619104</t>
+          <t>1.3522036001636815,0.08644916314895364,0.17935963607356278</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -882,11 +882,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.02178692856264347</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1,0.9968717931264877,0.7688099775153753</t>
+          <t>1.3522036001636815,0.011106346459674236,0.17935963607356278</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -895,11 +895,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.02178692856264347</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2.0799864236490704,0.9538647943932738,0.8863103755483714</t>
+          <t>1.3522036001636815,0.08644916314895364,0.17935963607356278</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -908,11 +908,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.02176399463641286</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1.8631259581568624,0.9727205942395488,0.9308227231670749</t>
+          <t>1.3390011457128044,0.1725594425881081,0.28665690314747894</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -921,11 +921,11 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.02176399463641286</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1.8631259581568624,0.9727205942395488,0.8482040870519428</t>
+          <t>1.2151721903156767,0.07260106292808893,0.15602401764696042</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -934,11 +934,11 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.02176399463641286</v>
+        <v>0.02470552189983371</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2.105783911668174,1.0471454871684038,0.45</t>
+          <t>1.632524302044787e-05,0.030475863507476195,6.974030110261142e-05</t>
         </is>
       </c>
       <c r="C21" t="n">

</xml_diff>

<commit_message>
added error calculation and testing, also some debugging (referencing)
</commit_message>
<xml_diff>
--- a/Scripts/Testing/Genetic_algorithm_tests/Results/toy_model_parametrization.xlsx
+++ b/Scripts/Testing/Genetic_algorithm_tests/Results/toy_model_parametrization.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="5">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.352203600163681</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.08644916314895364</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1793596360735628</v>
+        <v>0.45</v>
       </c>
     </row>
   </sheetData>
@@ -687,11 +687,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2.8924638724579337,0.569524159734011,1.6708405900886545</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -700,11 +700,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3.051938536522032,0.569524159734011,4.475213211331274</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -713,11 +713,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3.848845395901783,1.4365499502385757,0.20217472269133435</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -726,11 +726,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.987646918070706,0.2541695329592857,0.017097034978287927</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -739,11 +739,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.0062370479940266,0.0017002151129185455,0.08451912524871687</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -752,11 +752,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.2787626029336818,0.19496244078662248,1.4950900680884687</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -765,11 +765,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.5402939795689649,0.020983948799077404,0.27806590837091927</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -778,11 +778,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0.7392657256664663,2.4734802075819955,0.0030627848696714974</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -791,11 +791,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1.275396514892563,0.4782933443632343,3.0964047138813497</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -804,11 +804,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.03082930686377845</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.3817751388303598,0.01649286043169756,1.985586888796016</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -817,11 +817,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.4828720420349909,0.14892421624637012,0.2783129012578397</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -830,11 +830,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1.4324850413658867,0.0002021472584592835,0.02950125796447201</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -843,11 +843,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.365644485548155,1.3330180608434845,0.11536738791278571</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -856,11 +856,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1.4341642450747463,0.0033107260580177134,0.00025270797536693275</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -869,11 +869,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1.3522036001636815,0.08644916314895364,0.17935963607356278</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -882,11 +882,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1.3522036001636815,0.011106346459674236,0.17935963607356278</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -895,11 +895,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1.3522036001636815,0.08644916314895364,0.17935963607356278</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -908,11 +908,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1.3390011457128044,0.1725594425881081,0.28665690314747894</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -921,11 +921,11 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1.2151721903156767,0.07260106292808893,0.15602401764696042</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -934,11 +934,11 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.02470552189983371</v>
+        <v>0.02231684822881893</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1.632524302044787e-05,0.030475863507476195,6.974030110261142e-05</t>
+          <t>1,0.5,0.45</t>
         </is>
       </c>
       <c r="C21" t="n">

</xml_diff>

<commit_message>
fixed bug error calculation
</commit_message>
<xml_diff>
--- a/Scripts/Testing/Genetic_algorithm_tests/Results/toy_model_parametrization.xlsx
+++ b/Scripts/Testing/Genetic_algorithm_tests/Results/toy_model_parametrization.xlsx
@@ -451,7 +451,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.2028568963115664</v>
       </c>
     </row>
     <row r="3">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>0.4683441826985172</v>
       </c>
     </row>
     <row r="4">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.45</v>
+        <v>0.4609422306163425</v>
       </c>
     </row>
   </sheetData>
@@ -687,11 +687,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.03108594233577064</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.00041653920881596377,0.0010050439438327762,0.13581123877541385</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -700,11 +700,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>1.102397224308144,2.048150953236908,0.007377455110109631</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -713,11 +713,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>1.0270181763836395,0.35787412489103565,0.06278825883706389</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -726,11 +726,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.7430363133905642,2.1053482067252487,0.14013869955958885</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -739,11 +739,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.4303959341128161,0.4924628954743089,0.18989777506233108</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -752,11 +752,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.003707304566609032,0.062362616664958744,0.5245124644363194</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -765,11 +765,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>1,0.5986374499100555,0.13468878527787956</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -778,11 +778,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>1.168568553778462,0.2063330605685388,1.2636887416745217</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -791,11 +791,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.5494546944153037,0.26039180357557007,0.07700585918366556</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -804,11 +804,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.8902343836563613,0.6652486883233962,0.19813415730406841</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -817,11 +817,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02347670333605364</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.4399441635055259,0.5563933671383474,0.22930533011576582</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -830,11 +830,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.056338586123188504,0.10241493851108913,0.5935367995437807</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -843,11 +843,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.20833771971674991,0.27998292548557074,0.21487876681909404</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -856,11 +856,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.08924570755911927,0.33413009004765176,0.7847461846041075</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -869,11 +869,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.39456891523400117,0.46834418269851724,0.7003040914345592</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -882,11 +882,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.33831550135894867,1.2222372298753486,2.3387322170294187</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -895,11 +895,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.342711089771747,0.9914881140635853,0.0787847279145073</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -908,11 +908,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.16020245878542141,0.7464085486862838,1.1230351433705095</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -921,11 +921,11 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.061038578999222264,0.22961920006096267,0.33006968584244595</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -934,11 +934,11 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.02231684822881893</v>
+        <v>0.02291017914415097</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1,0.5,0.45</t>
+          <t>0.20285689631156636,0.46834418269851724,0.4609422306163425</t>
         </is>
       </c>
       <c r="C21" t="n">

</xml_diff>